<commit_message>
docs(data): add anonymized tester feedback dataset
</commit_message>
<xml_diff>
--- a/docs/data/stellar_shield_tester_feedback_anonymized.xlsx
+++ b/docs/data/stellar_shield_tester_feedback_anonymized.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="81">
   <si>
     <t>Zaman damgası</t>
   </si>
@@ -243,6 +243,21 @@
   </si>
   <si>
     <t>a408d3feee7ed166c3adc211be332a68a3a518876b68dda63de9782188cd99d3</t>
+  </si>
+  <si>
+    <t>Shubhajeet Saha</t>
+  </si>
+  <si>
+    <t>shubhajeetsaha26@gmail.com</t>
+  </si>
+  <si>
+    <t>GCJIUYSSF4CY33BNQGASBOMBCJWK5QXGDJB5F4ZPLSVHFJNMGEUPMNAU</t>
+  </si>
+  <si>
+    <t>Its all good, liked the website and all the features</t>
+  </si>
+  <si>
+    <t>f47d3aa98b898220b51a3e15f2791addb562d20496cf49d72caf3e86f9735628</t>
   </si>
 </sst>
 </file>
@@ -392,7 +407,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:M13" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:M14" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="13">
     <tableColumn name="Zaman damgası" id="1"/>
     <tableColumn name="Name " id="2"/>
@@ -614,7 +629,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="3" width="18.88"/>
-    <col customWidth="1" min="4" max="4" width="27.88"/>
+    <col customWidth="1" min="4" max="4" width="62.38"/>
     <col customWidth="1" min="5" max="9" width="37.63"/>
     <col customWidth="1" min="10" max="12" width="18.88"/>
     <col customWidth="1" min="13" max="13" width="37.63"/>
@@ -1051,6 +1066,38 @@
         <v>75</v>
       </c>
     </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="8">
+        <v>46262.80395700231</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>